<commit_message>
feat(artefacts): add story map v1.0
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-24-story-map-v1.0.xlsx
+++ b/docs/cadrage/equipe-24-story-map-v1.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/code/IPSSI_APOCAL_KIT/docs/cadrage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C536919D-88E0-1B4E-8C75-155106C5BBB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E948AD9-FB78-2546-B755-2BFAEB3FA094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -130,87 +130,15 @@
     <t>MUST : MVP Release 1</t>
   </si>
   <si>
-    <t>F1, Inscription email + mot de passe (Django Auth standard)</t>
-  </si>
-  <si>
-    <t>F2, Upload PDF ≤ 5 Mo OU saisie texte ≥ 200 caractères</t>
-  </si>
-  <si>
-    <t>F3, Génération automatique de 10 QCM via Llama 3.1 8B (Ollama local)</t>
-  </si>
-  <si>
-    <t>F4, Soumission + correction automatique (1 bonne réponse / QCM)</t>
-  </si>
-  <si>
-    <t>F5, Score /10 + détail des bonnes et mauvaises réponses</t>
-  </si>
-  <si>
-    <t>F6, Historique persistant des quizz par utilisateur</t>
-  </si>
-  <si>
     <t>SHOULD : Release 2</t>
   </si>
   <si>
-    <t>Reset password par email (lien magique 24 h)</t>
-  </si>
-  <si>
-    <t>Multi-cours (bibliothèque personnelle de cours uploadés)</t>
-  </si>
-  <si>
-    <t>Choix du niveau de difficulté + nombre de questions (5-20)</t>
-  </si>
-  <si>
-    <t>Mode timer optionnel par question (10-30 s configurable)</t>
-  </si>
-  <si>
-    <t>Dashboard progression par chapitre / cours</t>
-  </si>
-  <si>
-    <t>Export RGPD complet (JSON + CSV, Art. 15 / 20), lié J3-bis</t>
-  </si>
-  <si>
     <t>COULD : Release 2</t>
   </si>
   <si>
-    <t>Login social Google / Apple OAuth</t>
-  </si>
-  <si>
-    <t>Import d'un cours depuis une URL (article web, blog)</t>
-  </si>
-  <si>
-    <t>Mode questions ouvertes (correction LLM avec barème)</t>
-  </si>
-  <si>
-    <t>Mode flashcards type Anki (révision espacée)</t>
-  </si>
-  <si>
-    <t>Identification automatique des lacunes par chapitre</t>
-  </si>
-  <si>
-    <t>Suppression compte + données (RGPD Art. 17, droit à l'oubli)</t>
-  </si>
-  <si>
     <t>WON'T (this time)</t>
   </si>
   <si>
-    <t>SSO entreprise SAML / OIDC (B2B Release 3+)</t>
-  </si>
-  <si>
-    <t>Source vidéo ou audio (transcription Whisper coûteuse)</t>
-  </si>
-  <si>
-    <t>Compétition multi-joueurs (hors cible primaire)</t>
-  </si>
-  <si>
-    <t>Mode IA conversationnelle (chatbot type Khanmigo)</t>
-  </si>
-  <si>
-    <t>Stats temps réel collectives (besoin marginal MVP)</t>
-  </si>
-  <si>
-    <t>Personnalisation thème UI (thème sombre déjà imposé)</t>
-  </si>
-  <si>
     <t>📌 LÉGENDE</t>
   </si>
   <si>
@@ -302,6 +230,78 @@
   </si>
   <si>
     <t>Validé PO</t>
+  </si>
+  <si>
+    <t>US-01 Inscription email + mot de passe (Django Auth standard)</t>
+  </si>
+  <si>
+    <t>US-02 Upload PDF ≤ 5 Mo OU saisie texte ≥ 200 caractères</t>
+  </si>
+  <si>
+    <t>US-03 Génération automatique de 10 QCM via Llama 3.1 8B (Ollama local)</t>
+  </si>
+  <si>
+    <t>US-04 Soumission + correction automatique (1 bonne réponse / QCM)</t>
+  </si>
+  <si>
+    <t>US-05 Score /10 + détail des bonnes et mauvaises réponses</t>
+  </si>
+  <si>
+    <t>US-06 Historique persistant des quizz par utilisateur</t>
+  </si>
+  <si>
+    <t>US-07 Reset password par email (lien magique 24 h)</t>
+  </si>
+  <si>
+    <t>US-08 Multi-cours (bibliothèque personnelle de cours uploadés)</t>
+  </si>
+  <si>
+    <t>US-09 Choix du niveau de difficulté + nombre de questions (5-20)</t>
+  </si>
+  <si>
+    <t>US-10 Mode timer optionnel par question (10-30 s configurable)</t>
+  </si>
+  <si>
+    <t>US-11 Dashboard progression par chapitre / cours</t>
+  </si>
+  <si>
+    <t>US-12 Export RGPD complet (JSON + CSV, Art. 15 / 20), lié J3-bis</t>
+  </si>
+  <si>
+    <t>US-13 Login social Google / Apple OAuth</t>
+  </si>
+  <si>
+    <t>US- 14 Import d'un cours depuis une URL (article web, blog)</t>
+  </si>
+  <si>
+    <t>US-15 Mode questions ouvertes (correction LLM avec barème)</t>
+  </si>
+  <si>
+    <t>US- 16 Mode flashcards type Anki (révision espacée)</t>
+  </si>
+  <si>
+    <t>US- 17 Identification automatique des lacunes par chapitre</t>
+  </si>
+  <si>
+    <t>US- 18 Suppression compte + données (RGPD Art. 17, droit à l'oubli)</t>
+  </si>
+  <si>
+    <t>US-19 SSO entreprise SAML / OIDC (B2B Release 3+)</t>
+  </si>
+  <si>
+    <t>US-20 Source vidéo ou audio (transcription Whisper coûteuse)</t>
+  </si>
+  <si>
+    <t>US-21 Compétition multi-joueurs (hors cible primaire)</t>
+  </si>
+  <si>
+    <t>US-22 Mode IA conversationnelle (chatbot type Khanmigo)</t>
+  </si>
+  <si>
+    <t>US-23 Stats temps réel collectives (besoin marginal MVP)</t>
+  </si>
+  <si>
+    <t>US-24 Personnalisation thème UI (thème sombre déjà imposé)</t>
   </si>
 </sst>
 </file>
@@ -992,7 +992,7 @@
         <v>10</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1000,7 +1000,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1008,7 +1008,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1016,7 +1016,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
@@ -1024,7 +1024,7 @@
         <v>14</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
@@ -1121,136 +1121,136 @@
         <v>34</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>39</v>
+        <v>73</v>
       </c>
       <c r="G10" s="18" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B11" s="20" t="s">
-        <v>42</v>
+        <v>75</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>43</v>
+        <v>76</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>46</v>
+        <v>79</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>47</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>53</v>
+        <v>85</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>56</v>
+        <v>87</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="D13" s="24" t="s">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>61</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="26" t="s">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="28" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1271,104 +1271,104 @@
   <sheetData>
     <row r="2" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>73</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="16"/>
       <c r="B5" s="16" t="s">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>76</v>
+        <v>52</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="29" t="s">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="C6" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D6" s="29"/>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="29" t="s">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="C7" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D7" s="29"/>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="29" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="C8" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D8" s="29"/>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="29" t="s">
-        <v>82</v>
+        <v>58</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D9" s="29"/>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="29" t="s">
-        <v>83</v>
+        <v>59</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D10" s="29"/>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="29" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
       <c r="C11" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D11" s="29"/>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="29" t="s">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D12" s="29"/>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="29" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="C13" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D13" s="29"/>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="29" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="D14" s="29"/>
     </row>

</xml_diff>

<commit_message>
fix(artefacts): update story map pour reflect le product backlog
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-24-story-map-v1.0.xlsx
+++ b/docs/cadrage/equipe-24-story-map-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/code/IPSSI_APOCAL_KIT/docs/cadrage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E948AD9-FB78-2546-B755-2BFAEB3FA094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9DD2D8-3CA2-6A4F-A74F-B82601CCD426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,25 @@
     <sheet name="Story Map" sheetId="3" r:id="rId3"/>
     <sheet name="Auto-évaluation" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="94">
   <si>
     <t>A</t>
   </si>
@@ -286,22 +299,25 @@
     <t>US- 18 Suppression compte + données (RGPD Art. 17, droit à l'oubli)</t>
   </si>
   <si>
-    <t>US-19 SSO entreprise SAML / OIDC (B2B Release 3+)</t>
-  </si>
-  <si>
-    <t>US-20 Source vidéo ou audio (transcription Whisper coûteuse)</t>
-  </si>
-  <si>
-    <t>US-21 Compétition multi-joueurs (hors cible primaire)</t>
-  </si>
-  <si>
-    <t>US-22 Mode IA conversationnelle (chatbot type Khanmigo)</t>
-  </si>
-  <si>
-    <t>US-23 Stats temps réel collectives (besoin marginal MVP)</t>
-  </si>
-  <si>
-    <t>US-24 Personnalisation thème UI (thème sombre déjà imposé)</t>
+    <t>7. Encadrer sa classe</t>
+  </si>
+  <si>
+    <t>US-21 Créer une classe + inscrire des étudiants (S4) · US-22 Assigner un quiz via lien unique (S5)</t>
+  </si>
+  <si>
+    <t>US-23 Dashboard scores de la classe — moyenne + par étudiant (S6)</t>
+  </si>
+  <si>
+    <t>US-24 Repérer décrocheurs automatiquement · US-25 Envoyer conseil ciblé à un étudiant</t>
+  </si>
+  <si>
+    <t>US-18 SSO entreprise SAML/OIDC (B2B Release 3+)</t>
+  </si>
+  <si>
+    <t>US-19 Mode IA conversationnelle (chatbot type Khanmigo)</t>
+  </si>
+  <si>
+    <t>US-20 Compétition multi-joueurs (hors cible primaire)</t>
   </si>
 </sst>
 </file>
@@ -1044,24 +1060,24 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="7" width="32" customWidth="1"/>
+    <col min="2" max="8" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1069,7 +1085,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
@@ -1077,7 +1093,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>23</v>
       </c>
@@ -1085,7 +1101,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>25</v>
       </c>
@@ -1093,7 +1109,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="16" t="s">
         <v>27</v>
       </c>
@@ -1115,8 +1131,11 @@
       <c r="G9" s="16" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H9" s="16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="17" t="s">
         <v>34</v>
       </c>
@@ -1138,8 +1157,11 @@
       <c r="G10" s="18" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H10" s="18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
         <v>35</v>
       </c>
@@ -1161,8 +1183,11 @@
       <c r="G11" s="20" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H11" s="20" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
         <v>36</v>
       </c>
@@ -1184,36 +1209,34 @@
       <c r="G12" s="22" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="H12" s="22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="23" t="s">
         <v>37</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>88</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C13" s="24"/>
       <c r="D13" s="24" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>91</v>
-      </c>
-      <c r="G13" s="24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
         <v>39</v>
       </c>
@@ -1255,6 +1278,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>